<commit_message>
lab meeting schedule update
</commit_message>
<xml_diff>
--- a/lab_meeting/lab_meeting_calendar.xlsx
+++ b/lab_meeting/lab_meeting_calendar.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bcmedu-my.sharepoint.com/personal/u244834_bcm_edu/Documents/lab/websites/frankfort-lab/lab_meeting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="162" documentId="8_{B3463328-A060-409B-801D-1A35AED95DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F62E1F7D-A7EA-4095-92AF-7A1CCBB8E4DD}"/>
+  <xr:revisionPtr revIDLastSave="167" documentId="8_{B3463328-A060-409B-801D-1A35AED95DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9B543AF-E442-47B3-B031-AC022727E74B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{148D7F30-F220-420D-858E-D08D52631B38}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="56">
   <si>
     <t>Date</t>
   </si>
@@ -205,9 +205,6 @@
   </si>
   <si>
     <t>Reagan, Ritu, Miles, Molly, Grace</t>
-  </si>
-  <si>
-    <t>Ben Frankfort &amp; Daniel Brock</t>
   </si>
 </sst>
 </file>
@@ -1131,16 +1128,13 @@
         <v>46062</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1170,6 +1164,9 @@
       <c r="E8" t="b">
         <v>0</v>
       </c>
+      <c r="F8" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -1204,7 +1201,7 @@
         <v>46097</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>

</xml_diff>